<commit_message>
Daily EOD data and reports for 2026-10-19
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261019.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261019.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.76</v>
+        <v>1.745</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.02</v>
+        <v>-0.035</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-1.12%</t>
+          <t>-1.97%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>269598.56</v>
+        <v>267300.85</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-3063.62</v>
+        <v>-5361.33</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.415</v>
+        <v>2.445</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.035</v>
+        <v>0.065</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.47%</t>
+          <t>2.73%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>169050</v>
+        <v>171150</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>2450</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>60.1</v>
+        <v>60.37</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.34</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.12%</t>
+          <t>0.57%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>480800</v>
+        <v>482960</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>560</v>
+        <v>2720</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.001</v>
+        <v>-0.002</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-16.67%</t>
+          <t>-33.33%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>220.45</v>
+        <v>176.36</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-44.09</v>
+        <v>-88.18000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>155.35</v>
+        <v>155.77</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.97</v>
+        <v>1.39</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.63%</t>
+          <t>0.90%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.825</v>
+        <v>0.835</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.015</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-2.94%</t>
+          <t>-1.76%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>8250</v>
+        <v>8350</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-250</v>
+        <v>-150</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>194.485</v>
+        <v>193.55</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2.285</v>
+        <v>1.35</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.19%</t>
+          <t>0.70%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>777940</v>
+        <v>774200</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>9140</v>
+        <v>5400</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.215</v>
+        <v>0.22</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.01</v>
+        <v>-0.005</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-4.44%</t>
+          <t>-2.22%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>4300</v>
+        <v>4400</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-200</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>11.87</v>
+        <v>11.97</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.06</v>
+        <v>0.04</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.50%</t>
+          <t>0.34%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>36144.15</v>
+        <v>36448.65</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-182.7</v>
+        <v>121.8</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.078</v>
+        <v>0.002</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>2.56%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>752.96</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-734.14</v>
+        <v>18.82</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.095</v>
+        <v>-0.01</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-10.53%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>510</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-570</v>
+        <v>-60</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>35.37</v>
+        <v>35.415</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.22</v>
+        <v>0.265</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.63%</t>
+          <t>0.75%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.84</v>
+        <v>33.99</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2.11%</t>
+          <t>2.56%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>43585.92</v>
+        <v>43779.12</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>901.6</v>
+        <v>1094.8</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1789889.08</v>
+        <v>1790027.94</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>6607.05</v>
+        <v>6745.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>